<commit_message>
File 29 Jul SiteIQ pulls (FK505 now in the register; STOCKTAKE still to come)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0116SzhKPYLMjCEssbRpxP9L
</commit_message>
<xml_diff>
--- a/01_Reporting_Suite/Data_SiteIQ/DAILY_SUMMARY.xlsx
+++ b/01_Reporting_Suite/Data_SiteIQ/DAILY_SUMMARY.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="35">
   <si>
     <t>PROJECT SCHEDULE</t>
   </si>
@@ -33,10 +33,10 @@
     <t>Gladstone k2 2026 Shutdown</t>
   </si>
   <si>
-    <t>13/07/2026 01:07 PM</t>
-  </si>
-  <si>
-    <t>27/07/2026 01:07 PM</t>
+    <t>13/07/2026 05:42 AM</t>
+  </si>
+  <si>
+    <t>29/07/2026 05:42 AM</t>
   </si>
   <si>
     <t>Andrew Fisher</t>
@@ -112,6 +112,9 @@
   </si>
   <si>
     <t>TOTAL FOR: 26/07/2026</t>
+  </si>
+  <si>
+    <t>TOTAL FOR: 27/07/2026</t>
   </si>
   <si>
     <t>REPORT TOTAL:</t>
@@ -164,8 +167,8 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="27.1918983459473" customWidth="1"/>
-    <col min="2" max="2" width="20.7179412841797" customWidth="1"/>
-    <col min="3" max="3" width="20.7179412841797" customWidth="1"/>
+    <col min="2" max="2" width="20.8519611358643" customWidth="1"/>
+    <col min="3" max="3" width="20.8519611358643" customWidth="1"/>
     <col min="4" max="4" width="15.2527256011963" customWidth="1"/>
     <col min="5" max="5" width="35.4623603820801" customWidth="1"/>
   </cols>
@@ -211,11 +214,11 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:M13"/>
+  <dimension ref="A1:M14"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="22.6638088226318" customWidth="1"/>
-    <col min="2" max="2" width="9.140625" customWidth="1"/>
+    <col min="2" max="2" width="9.6135892868042" customWidth="1"/>
     <col min="3" max="3" width="12.0372314453125" customWidth="1"/>
     <col min="4" max="4" width="9.140625" customWidth="1"/>
     <col min="5" max="5" width="9.140625" customWidth="1"/>
@@ -726,40 +729,81 @@
         <v>33</v>
       </c>
       <c r="B13" s="0">
-        <v>64606.9</v>
+        <v>10324.67</v>
       </c>
       <c r="C13" s="0">
+        <v>0</v>
+      </c>
+      <c r="D13" s="0">
+        <v>0</v>
+      </c>
+      <c r="E13" s="0">
+        <v>0</v>
+      </c>
+      <c r="F13" s="0">
+        <v>0</v>
+      </c>
+      <c r="G13" s="0">
+        <v>0</v>
+      </c>
+      <c r="H13" s="0">
+        <v>0</v>
+      </c>
+      <c r="I13" s="0">
+        <v>0</v>
+      </c>
+      <c r="J13" s="0">
+        <v>0</v>
+      </c>
+      <c r="K13" s="0">
+        <v>0</v>
+      </c>
+      <c r="L13" s="0">
+        <v>0</v>
+      </c>
+      <c r="M13" s="0">
+        <v>10324.67</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="0" t="s">
+        <v>34</v>
+      </c>
+      <c r="B14" s="0">
+        <v>74931.57</v>
+      </c>
+      <c r="C14" s="0">
         <v>45000</v>
       </c>
-      <c r="D13" s="0">
+      <c r="D14" s="0">
         <v>58520</v>
       </c>
-      <c r="E13" s="0">
+      <c r="E14" s="0">
         <v>15605</v>
       </c>
-      <c r="F13" s="0">
-        <v>0</v>
-      </c>
-      <c r="G13" s="0">
-        <v>0</v>
-      </c>
-      <c r="H13" s="0">
-        <v>0</v>
-      </c>
-      <c r="I13" s="0">
-        <v>0</v>
-      </c>
-      <c r="J13" s="0">
-        <v>0</v>
-      </c>
-      <c r="K13" s="0">
-        <v>0</v>
-      </c>
-      <c r="L13" s="0">
-        <v>0</v>
-      </c>
-      <c r="M13" s="0">
-        <v>183731.9</v>
+      <c r="F14" s="0">
+        <v>0</v>
+      </c>
+      <c r="G14" s="0">
+        <v>0</v>
+      </c>
+      <c r="H14" s="0">
+        <v>0</v>
+      </c>
+      <c r="I14" s="0">
+        <v>0</v>
+      </c>
+      <c r="J14" s="0">
+        <v>0</v>
+      </c>
+      <c r="K14" s="0">
+        <v>0</v>
+      </c>
+      <c r="L14" s="0">
+        <v>0</v>
+      </c>
+      <c r="M14" s="0">
+        <v>194056.57</v>
       </c>
     </row>
   </sheetData>

</xml_diff>